<commit_message>
Sincronizacion 2026-09-28: cobertura (tres laminas y glosario), migracion interna neta (cinco laminas, por cada 1.000), mapas comunales de migracion desde la capa, dependencia/envejecimiento/otras relaciones con el diseno nuevo, ingresos semestral con total nacional
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/graficos_dimensiones/comunal_m_miginterna_a_2019_antofagasta.xlsx
+++ b/output/graficos_dimensiones/comunal_m_miginterna_a_2019_antofagasta.xlsx
@@ -69,7 +69,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-24 00:26</t>
+    <t xml:space="preserve">2026-09-27 23:09</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -505,7 +505,7 @@
         <v>2019</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>7.62</v>
+        <v>76.24</v>
       </c>
     </row>
     <row r="3">
@@ -522,7 +522,7 @@
         <v>2019</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>5.7</v>
+        <v>56.99</v>
       </c>
     </row>
     <row r="4">
@@ -539,7 +539,7 @@
         <v>2019</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.88</v>
+        <v>8.76</v>
       </c>
     </row>
     <row r="5">
@@ -573,7 +573,7 @@
         <v>2019</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-0.14</v>
+        <v>-1.44</v>
       </c>
     </row>
     <row r="7">
@@ -590,7 +590,7 @@
         <v>2019</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-0.18</v>
+        <v>-1.77</v>
       </c>
     </row>
     <row r="8">
@@ -607,7 +607,7 @@
         <v>2019</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-0.25</v>
+        <v>-2.53</v>
       </c>
     </row>
     <row r="9">
@@ -624,7 +624,7 @@
         <v>2019</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-1.33</v>
+        <v>-13.33</v>
       </c>
     </row>
     <row r="10">
@@ -641,7 +641,7 @@
         <v>2019</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-1.69</v>
+        <v>-16.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>